<commit_message>
vars update, new evals, small refactors
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -307,7 +307,7 @@
     <t>Levels</t>
   </si>
   <si>
-    <t>6, 7, 8, 9, 10, 11, 12</t>
+    <t>6, 7, 8, 9, 10, 11, 12, 13, 14</t>
   </si>
   <si>
     <r>
@@ -1014,7 +1014,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1025,12 +1025,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1068,7 +1062,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1076,20 +1070,14 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,56 +1384,56 @@
   <dimension ref="A1:AX3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="6" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="6" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="6" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="6" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="6" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="6" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="6" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="6" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="6" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="6" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="6" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="6" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="44" max="44" style="6" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="45" max="45" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="46" max="46" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="47" max="47" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="48" max="48" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="49" max="49" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="50" max="50" style="7" width="24.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="5" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="5" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="5" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="5" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="5" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="5" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="5" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="5" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="5" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="5" width="24.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
@@ -1497,10 +1485,10 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="2" t="s">
@@ -1524,10 +1512,10 @@
       <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
       <c r="AB1" s="2" t="s">
@@ -1647,10 +1635,10 @@
       <c r="P2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>65</v>
       </c>
       <c r="S2" s="2" t="s">
@@ -1674,13 +1662,13 @@
       <c r="Y2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="Z2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AA2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AB2" s="2" t="s">
         <v>75</v>
       </c>
       <c r="AC2" s="2" t="s">
@@ -1759,7 +1747,7 @@
         <v>97</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="4"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -1779,16 +1767,16 @@
       <c r="N3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="O3" s="4" t="s">
         <v>103</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Q3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" s="2" t="s">
         <v>106</v>
       </c>
       <c r="S3" s="2"/>
@@ -1850,7 +1838,7 @@
         <v>114</v>
       </c>
       <c r="AW3" s="2"/>
-      <c r="AX3" s="3"/>
+      <c r="AX3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
vars update, new evals, small refactors (#539)
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
+++ b/dashboard-ui/src/components/SurveyResults/Survey Delegation Variables - PH2.xlsx
@@ -307,7 +307,7 @@
     <t>Levels</t>
   </si>
   <si>
-    <t>6, 7, 8, 9, 10, 11, 12</t>
+    <t>6, 7, 8, 9, 10, 11, 12, 13, 14</t>
   </si>
   <si>
     <r>
@@ -1014,7 +1014,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1025,12 +1025,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1068,7 +1062,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1076,20 +1070,14 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,56 +1384,56 @@
   <dimension ref="A1:AX3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="7" width="14.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="7" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="6" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="6" width="20.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="6" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="6" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="6" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="6" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="6" width="18.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="6" width="18.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="6" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="6" width="16.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="6" width="24.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="6" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="6" width="25.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="6" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="6" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="6" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="44" max="44" style="6" width="25.005" customWidth="1" bestFit="1"/>
-    <col min="45" max="45" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="46" max="46" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="47" max="47" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="48" max="48" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="49" max="49" style="6" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="50" max="50" style="7" width="24.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="14.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="5" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="5" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="5" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="5" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="5" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="5" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="5" width="16.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="5" width="24.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="5" width="22.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="5" width="25.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="5" width="18.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="5" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="5" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="5" width="25.005" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="5" width="32.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="5" width="24.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="73.5" customFormat="1" s="1">
@@ -1497,10 +1485,10 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="2" t="s">
@@ -1524,10 +1512,10 @@
       <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
       <c r="AB1" s="2" t="s">
@@ -1647,10 +1635,10 @@
       <c r="P2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>65</v>
       </c>
       <c r="S2" s="2" t="s">
@@ -1674,13 +1662,13 @@
       <c r="Y2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Z2" s="3" t="s">
+      <c r="Z2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AA2" s="3" t="s">
+      <c r="AA2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AB2" s="2" t="s">
         <v>75</v>
       </c>
       <c r="AC2" s="2" t="s">
@@ -1759,7 +1747,7 @@
         <v>97</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="4"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -1779,16 +1767,16 @@
       <c r="N3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="O3" s="4" t="s">
         <v>103</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Q3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" s="2" t="s">
         <v>106</v>
       </c>
       <c r="S3" s="2"/>
@@ -1850,7 +1838,7 @@
         <v>114</v>
       </c>
       <c r="AW3" s="2"/>
-      <c r="AX3" s="3"/>
+      <c r="AX3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>